<commit_message>
Reposiciona business plan para tese dupla (defensiva Coaph + ofensiva)
- Reframe de "marketplace nacional" para "automação operacional da Coaph,
  com opção de escalar". Decisão ancorada na economia operacional, não na
  escala externa.
- Modelo financeiro: nova aba "ROI Coaph" (custo R$240k/mês, payback por
  % de economia, ROI) separada da receita da startup. 112 fórmulas, 0 erros.
- Business plan: novas seções (tese, business case Coaph, KPIs do piloto,
  recomendação trancheada); riscos ampliados; tom mais maduro.
- Pitch deck: 5 slides novos (tese dupla, ROI Coaph, pior cenário, tranches,
  KPIs); mercado/projeções remarcados como upside.
- Novos entregáveis: one-pager para a diretoria (1 pág) e recomendação
  brutalmente honesta de quando investir e quando não.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/business-plan/HealthMatch_Modelo_Financeiro.xlsx
+++ b/business-plan/HealthMatch_Modelo_Financeiro.xlsx
@@ -9,10 +9,11 @@
   </bookViews>
   <sheets>
     <sheet name="Premissas" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Cenários" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="DRE (Realista)" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Métricas" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Uso dos Recursos" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="ROI Coaph" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Cenários" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="DRE (Realista)" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Métricas" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Uso dos Recursos" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="95">
   <si>
     <t xml:space="preserve">HealthMatch — Modelo Financeiro (Pre-seed)</t>
   </si>
@@ -102,6 +103,51 @@
   </si>
   <si>
     <t xml:space="preserve">Opex total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROI Coaph — Economia Operacional (tese defensiva)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economia na operação da PRÓPRIA Coaph ao automatizar a gestão de plantões. NÃO é receita do HealthMatch — é a justificativa estratégica do investimento pela Coaph (paga-se mesmo sem escala externa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premissas (editáveis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custo atual/mês com prepostos e operação manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Investimento total (pre-seed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custo anual atual com prepostos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cenários de economia → payback do investimento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% economia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economia/mês</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economia/ano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payback (meses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROI anual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teto teórico (não usar como base)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base de defesa do investimento: 25% (conservador) a 50% (realista). 100% é teto teórico — exigiria redesenho operacional total e NÃO deve ser premissa-base.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importante: esta economia NÃO se soma à receita do HealthMatch (abas Cenários/DRE). São lentes distintas — a economia justifica o aporte da Coaph; a receita é o upside da escala externa.</t>
   </si>
   <si>
     <t xml:space="preserve">Projeção de receita — 3 cenários</t>
@@ -437,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -486,6 +532,30 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -498,15 +568,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1151,6 +1213,238 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <f aca="false">B5*12</f>
+        <v>2880000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <f aca="false">$B$5*B11</f>
+        <v>60000</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <f aca="false">C11*12</f>
+        <v>720000</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <f aca="false">$B$6/C11</f>
+        <v>25</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <f aca="false">D11/$B$6</f>
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <f aca="false">$B$5*B12</f>
+        <v>120000</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <f aca="false">C12*12</f>
+        <v>1440000</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <f aca="false">$B$6/C12</f>
+        <v>12.5</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <f aca="false">D12/$B$6</f>
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <f aca="false">$B$5*B13</f>
+        <v>180000</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <f aca="false">C13*12</f>
+        <v>2160000</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <f aca="false">$B$6/C13</f>
+        <v>8.33333333333333</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <f aca="false">D13/$B$6</f>
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <f aca="false">$B$5*B14</f>
+        <v>240000</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <f aca="false">C14*12</f>
+        <v>2880000</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <f aca="false">$B$6/C14</f>
+        <v>6.25</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <f aca="false">D14/$B$6</f>
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1161,7 +1455,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1171,7 +1465,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1181,81 +1475,81 @@
       <c r="G2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="13" t="s">
+      <c r="A5" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="19" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="B6" s="20" t="n">
         <f aca="false">Premissas!C13*Premissas!$B$8*Premissas!$B$5</f>
         <v>6240000</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="20" t="n">
         <f aca="false">Premissas!D13*Premissas!$B$8*Premissas!$B$5</f>
         <v>34320000</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="20" t="n">
         <f aca="false">Premissas!E13*Premissas!$B$8*Premissas!$B$5</f>
         <v>93600000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B7" s="13" t="n">
         <f aca="false">B6*Premissas!C16</f>
         <v>312000</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="13" t="n">
         <f aca="false">C6*Premissas!D16</f>
         <v>1716000</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="13" t="n">
         <f aca="false">D6*Premissas!E16</f>
         <v>4680000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B8" s="20" t="n">
         <f aca="false">Premissas!C19*Premissas!$B$6*Premissas!$B$8</f>
         <v>120000</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="20" t="n">
         <f aca="false">Premissas!D19*Premissas!$B$6*Premissas!$B$8</f>
         <v>540000</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="20" t="n">
         <f aca="false">Premissas!E19*Premissas!$B$6*Premissas!$B$8</f>
         <v>1700160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">B7+B8</f>
@@ -1271,81 +1565,81 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="13" t="s">
+      <c r="A12" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="19" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="B13" s="20" t="n">
         <f aca="false">Premissas!C14*Premissas!$B$8*Premissas!$B$5</f>
         <v>12480000</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="20" t="n">
         <f aca="false">Premissas!D14*Premissas!$B$8*Premissas!$B$5</f>
         <v>70200000</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="20" t="n">
         <f aca="false">Premissas!E14*Premissas!$B$8*Premissas!$B$5</f>
         <v>187200000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B14" s="13" t="n">
         <f aca="false">B13*Premissas!C17</f>
         <v>873600</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="13" t="n">
         <f aca="false">C13*Premissas!D17</f>
         <v>4914000</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">D13*Premissas!E17</f>
         <v>13104000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B15" s="20" t="n">
         <f aca="false">Premissas!C20*Premissas!$B$6*Premissas!$B$8</f>
         <v>216000</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="20" t="n">
         <f aca="false">Premissas!D20*Premissas!$B$6*Premissas!$B$8</f>
         <v>1080000</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="20" t="n">
         <f aca="false">Premissas!E20*Premissas!$B$6*Premissas!$B$8</f>
         <v>3360000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">B14+B15</f>
@@ -1361,81 +1655,81 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="13" t="s">
+      <c r="A19" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="19" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="B20" s="20" t="n">
         <f aca="false">Premissas!C15*Premissas!$B$8*Premissas!$B$5</f>
         <v>20280000</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="20" t="n">
         <f aca="false">Premissas!D15*Premissas!$B$8*Premissas!$B$5</f>
         <v>124800000</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="20" t="n">
         <f aca="false">Premissas!E15*Premissas!$B$8*Premissas!$B$5</f>
         <v>343200000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B21" s="13" t="n">
         <f aca="false">B20*Premissas!C18</f>
         <v>1622400</v>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="13" t="n">
         <f aca="false">C20*Premissas!D18</f>
         <v>9984000</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="13" t="n">
         <f aca="false">D20*Premissas!E18</f>
         <v>27456000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B22" s="20" t="n">
         <f aca="false">Premissas!C21*Premissas!$B$6*Premissas!$B$8</f>
         <v>360000</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="20" t="n">
         <f aca="false">Premissas!D21*Premissas!$B$6*Premissas!$B$8</f>
         <v>1899840</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="20" t="n">
         <f aca="false">Premissas!E21*Premissas!$B$6*Premissas!$B$8</f>
         <v>5799840</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B23" s="11" t="n">
         <f aca="false">B21+B22</f>
@@ -1452,23 +1746,23 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="19" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1476,15 +1770,15 @@
       <c r="A26" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="16" t="n">
+      <c r="B26" s="21" t="n">
         <f aca="false">B9</f>
         <v>432000</v>
       </c>
-      <c r="C26" s="16" t="n">
+      <c r="C26" s="21" t="n">
         <f aca="false">C9</f>
         <v>2256000</v>
       </c>
-      <c r="D26" s="16" t="n">
+      <c r="D26" s="21" t="n">
         <f aca="false">D9</f>
         <v>6380160</v>
       </c>
@@ -1493,15 +1787,15 @@
       <c r="A27" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="16" t="n">
+      <c r="B27" s="21" t="n">
         <f aca="false">B16</f>
         <v>1089600</v>
       </c>
-      <c r="C27" s="16" t="n">
+      <c r="C27" s="21" t="n">
         <f aca="false">C16</f>
         <v>5994000</v>
       </c>
-      <c r="D27" s="16" t="n">
+      <c r="D27" s="21" t="n">
         <f aca="false">D16</f>
         <v>16464000</v>
       </c>
@@ -1510,15 +1804,15 @@
       <c r="A28" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="16" t="n">
+      <c r="B28" s="21" t="n">
         <f aca="false">B23</f>
         <v>1982400</v>
       </c>
-      <c r="C28" s="16" t="n">
+      <c r="C28" s="21" t="n">
         <f aca="false">C23</f>
         <v>11883840</v>
       </c>
-      <c r="D28" s="16" t="n">
+      <c r="D28" s="21" t="n">
         <f aca="false">D23</f>
         <v>33255840</v>
       </c>
@@ -1542,7 +1836,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1557,7 +1851,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1566,7 +1860,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1575,7 +1869,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -1589,41 +1883,41 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="B5" s="20" t="n">
         <f aca="false">Cenários!B16</f>
         <v>1089600</v>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="20" t="n">
         <f aca="false">Cenários!C16</f>
         <v>5994000</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="20" t="n">
         <f aca="false">Cenários!D16</f>
         <v>16464000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="15" t="n">
+        <v>53</v>
+      </c>
+      <c r="B6" s="13" t="n">
         <f aca="false">-B5*(1-Premissas!$B$7)</f>
         <v>-348672</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="13" t="n">
         <f aca="false">-C5*(1-Premissas!$B$7)</f>
         <v>-1918080</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="13" t="n">
         <f aca="false">-D5*(1-Premissas!$B$7)</f>
         <v>-5268480</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">B5+B6</f>
@@ -1640,85 +1934,85 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="17" t="n">
+        <v>55</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <f aca="false">B7/B5</f>
         <v>0.68</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="15" t="n">
         <f aca="false">C7/C5</f>
         <v>0.68</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="15" t="n">
         <f aca="false">D7/D5</f>
         <v>0.68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <f aca="false">-Premissas!C25</f>
         <v>-1100000</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="20" t="n">
         <f aca="false">-Premissas!D25</f>
         <v>-2400000</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="20" t="n">
         <f aca="false">-Premissas!E25</f>
         <v>-4800000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="14" t="n">
+        <v>57</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <f aca="false">-Premissas!C26</f>
         <v>-150000</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="20" t="n">
         <f aca="false">-Premissas!D26</f>
         <v>-600000</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="20" t="n">
         <f aca="false">-Premissas!E26</f>
         <v>-1800000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="B11" s="20" t="n">
         <f aca="false">-Premissas!C27</f>
         <v>-120000</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="20" t="n">
         <f aca="false">-Premissas!D27</f>
         <v>-300000</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="20" t="n">
         <f aca="false">-Premissas!E27</f>
         <v>-700000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="B12" s="20" t="n">
         <f aca="false">-Premissas!C28</f>
         <v>-120000</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="20" t="n">
         <f aca="false">-Premissas!D28</f>
         <v>-300000</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="20" t="n">
         <f aca="false">-Premissas!E28</f>
         <v>-700000</v>
       </c>
@@ -1741,35 +2035,35 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="18" t="n">
+      <c r="A14" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="22" t="n">
         <f aca="false">B7+B13</f>
         <v>-749072</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">C7+C13</f>
         <v>475920.000000001</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="22" t="n">
         <f aca="false">D7+D13</f>
         <v>3195520</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <f aca="false">B14/B5</f>
         <v>-0.687474302496329</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="15" t="n">
         <f aca="false">C14/C5</f>
         <v>0.0793993993993995</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="15" t="n">
         <f aca="false">D14/D5</f>
         <v>0.194091350826045</v>
       </c>
@@ -1789,7 +2083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1805,7 +2099,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1813,7 +2107,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1822,99 +2116,99 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>66</v>
+      </c>
+      <c r="B5" s="20" t="n">
         <f aca="false">Premissas!$B$6</f>
         <v>4000</v>
       </c>
-      <c r="C5" s="19" t="s">
-        <v>52</v>
+      <c r="C5" s="23" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>0.8</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>54</v>
+      <c r="C6" s="23" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>15000</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>56</v>
+      <c r="C7" s="23" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>0.12</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>54</v>
+      <c r="C8" s="23" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="C9" s="19" t="s">
-        <v>59</v>
+      <c r="C9" s="23" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="17" t="n">
+        <v>76</v>
+      </c>
+      <c r="B12" s="15" t="n">
         <f aca="false">1-(1-B8)^(1/12)</f>
         <v>0.010596241035319</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="15" t="n">
+        <v>77</v>
+      </c>
+      <c r="B13" s="13" t="n">
         <f aca="false">B5*B6</f>
         <v>3200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">B13*B9</f>
@@ -1922,32 +2216,32 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="20" t="n">
+      <c r="A15" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="24" t="n">
         <f aca="false">B14/B7</f>
         <v>7.68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="21" t="n">
+        <v>80</v>
+      </c>
+      <c r="B16" s="25" t="n">
         <f aca="false">B7/B13</f>
         <v>4.6875</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>67</v>
+      <c r="C18" s="23" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1966,7 +2260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1982,7 +2276,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1990,7 +2284,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>1500000</v>
@@ -1998,80 +2292,80 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>0.55</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="13" t="n">
         <f aca="false">$B$3*B6</f>
         <v>825000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>0.18</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="13" t="n">
         <f aca="false">$B$3*B7</f>
         <v>270000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="13" t="n">
         <f aca="false">$B$3*B8</f>
         <v>150000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="B9" s="6" t="n">
         <v>0.09</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="13" t="n">
         <f aca="false">$B$3*B9</f>
         <v>135000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>0.08</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="13" t="n">
         <f aca="false">$B$3*B10</f>
         <v>120000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="22" t="n">
+        <v>92</v>
+      </c>
+      <c r="B11" s="26" t="n">
         <f aca="false">SUM(B6:B10)</f>
         <v>1</v>
       </c>
@@ -2082,7 +2376,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>20</v>
@@ -2090,9 +2384,9 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="B14" s="20" t="n">
         <f aca="false">'DRE (Realista)'!B14</f>
         <v>-749072</v>
       </c>

</xml_diff>